<commit_message>
v0.2 — full dashboard rebuild + pipeline fixes
- Rebuilt app.py: 7 pages, MASI KPIs, metric explorer, heatmap, rolling vol/drawdown/histogram, portfolio evolution charts, full screener
- Fixed daily_automation.py: parse date index as Timestamp (DateOffset arithmetic was failing)
- Fixed run_daily.bat: create logs/ folder, copy outputs to data/ for Streamlit
- Registered Task Scheduler task (weekdays 09:00)
- Updated data files to 2026-04-15

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/portfolio_metrics_latest.xlsx
+++ b/data/portfolio_metrics_latest.xlsx
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3547"/>
+  <dimension ref="A1:B3549"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -35961,6 +35961,26 @@
       </c>
       <c r="B3547" s="3" t="n">
         <v>-0.504935</v>
+      </c>
+    </row>
+    <row r="3548">
+      <c r="A3548" s="2" t="inlineStr">
+        <is>
+          <t>14/04/2026</t>
+        </is>
+      </c>
+      <c r="B3548" s="2" t="n">
+        <v>2.151144</v>
+      </c>
+    </row>
+    <row r="3549">
+      <c r="A3549" s="3" t="inlineStr">
+        <is>
+          <t>15/04/2026</t>
+        </is>
+      </c>
+      <c r="B3549" s="3" t="n">
+        <v>1.033752</v>
       </c>
     </row>
   </sheetData>
@@ -35999,27 +36019,27 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>1Y  (2025-04-13 to 2026-04-13)</t>
+          <t>1Y  (2025-04-15 to 2026-04-15)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>2Y  (2024-04-13 to 2026-04-13)</t>
+          <t>2Y  (2024-04-15 to 2026-04-15)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>3Y  (2023-04-13 to 2026-04-13)</t>
+          <t>3Y  (2023-04-15 to 2026-04-15)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>4Y  (2022-04-13 to 2026-04-13)</t>
+          <t>4Y  (2022-04-15 to 2026-04-15)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>5Y  (2021-04-13 to 2026-04-13)</t>
+          <t>5Y  (2021-04-15 to 2026-04-15)</t>
         </is>
       </c>
     </row>
@@ -36035,19 +36055,19 @@
         </is>
       </c>
       <c r="C2" s="5" t="n">
-        <v>18.239</v>
+        <v>18.0531</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>15.7699</v>
+        <v>15.8079</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>13.9786</v>
+        <v>14.029</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>13.6478</v>
+        <v>13.6893</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>12.9406</v>
+        <v>12.9754</v>
       </c>
     </row>
     <row r="3">
@@ -36062,19 +36082,19 @@
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>18.0869</v>
+        <v>17.9309</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>15.9765</v>
+        <v>16.0236</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>14.1104</v>
+        <v>14.1672</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>13.6404</v>
+        <v>13.6884</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>13.0102</v>
+        <v>13.0505</v>
       </c>
     </row>
     <row r="5">
@@ -36089,19 +36109,19 @@
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>14.4706</v>
+        <v>13.5222</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>17.7247</v>
+        <v>19.0689</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>20.9864</v>
+        <v>22.0542</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>9.184200000000001</v>
+        <v>9.840400000000001</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>9.6989</v>
+        <v>10.2193</v>
       </c>
     </row>
     <row r="6">
@@ -36116,19 +36136,19 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>23.8257</v>
+        <v>23.7922</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>31.7775</v>
+        <v>33.7672</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>33.2925</v>
+        <v>34.7481</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>19.8795</v>
+        <v>20.8899</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>20.274</v>
+        <v>20.9463</v>
       </c>
     </row>
     <row r="8">
@@ -36143,19 +36163,19 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>0.6671</v>
+        <v>0.621</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>0.8057</v>
+        <v>0.8875</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.9144</v>
+        <v>0.9876</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>-0.1095</v>
+        <v>-0.0616</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>-0.2093</v>
+        <v>-0.1692</v>
       </c>
     </row>
     <row r="9">
@@ -36170,19 +36190,19 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>1.19</v>
+        <v>1.1979</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>1.6748</v>
+        <v>1.7929</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>1.778</v>
+        <v>1.8739</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>0.6746</v>
+        <v>0.7456</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>0.6047</v>
+        <v>0.6538</v>
       </c>
     </row>
     <row r="11">
@@ -36224,19 +36244,19 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>0.9799</v>
+        <v>0.9802999999999999</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>0.9969</v>
+        <v>0.997</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>0.9845</v>
+        <v>0.9846</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>0.9697</v>
+        <v>0.97</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>0.9721</v>
+        <v>0.9724</v>
       </c>
     </row>
     <row r="14">
@@ -36278,19 +36298,19 @@
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>2.805</v>
+        <v>2.9045</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>2.8448</v>
+        <v>2.8901</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>3.124</v>
+        <v>3.1531</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>3.3279</v>
+        <v>3.3492</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>3.337</v>
+        <v>3.3529</v>
       </c>
     </row>
     <row r="17">
@@ -36317,7 +36337,7 @@
         <v>0</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -36332,19 +36352,19 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>0.096</v>
+        <v>0.1049</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>0.1409</v>
+        <v>0.1474</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>0.125</v>
+        <v>0.1291</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>0.1065</v>
+        <v>0.1102</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>0.105</v>
+        <v>0.1067</v>
       </c>
     </row>
     <row r="20">
@@ -36413,10 +36433,10 @@
         </is>
       </c>
       <c r="C23" s="5" t="n">
-        <v>1.5293</v>
+        <v>1.5288</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>1.2846</v>
+        <v>1.2823</v>
       </c>
       <c r="E23" s="5" t="n">
         <v>1.1344</v>
@@ -36440,10 +36460,10 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>1.5417</v>
+        <v>1.541</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>1.2942</v>
+        <v>1.2924</v>
       </c>
       <c r="E24" s="7" t="n">
         <v>1.1507</v>
@@ -36521,19 +36541,19 @@
         </is>
       </c>
       <c r="C29" s="5" t="n">
-        <v>0.9673</v>
+        <v>0.8929</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>1.1502</v>
+        <v>1.2727</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>1.3595</v>
+        <v>1.4739</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>-0.1555</v>
+        <v>-0.0878</v>
       </c>
       <c r="G29" s="5" t="n">
-        <v>-0.2954</v>
+        <v>-0.2394</v>
       </c>
     </row>
     <row r="30">
@@ -36548,19 +36568,19 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>1.7698</v>
+        <v>1.7699</v>
       </c>
       <c r="D30" s="7" t="n">
-        <v>2.4703</v>
+        <v>2.6576</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>2.7249</v>
+        <v>2.8842</v>
       </c>
       <c r="F30" s="7" t="n">
-        <v>0.9859</v>
+        <v>1.0935</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>0.8766</v>
+        <v>0.9507</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Data update to 2026-04-21 + add Annualized Variance metric
</commit_message>
<xml_diff>
--- a/data/portfolio_metrics_latest.xlsx
+++ b/data/portfolio_metrics_latest.xlsx
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3549"/>
+  <dimension ref="A1:B3553"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -35981,6 +35981,46 @@
       </c>
       <c r="B3549" s="3" t="n">
         <v>1.033752</v>
+      </c>
+    </row>
+    <row r="3550">
+      <c r="A3550" s="2" t="inlineStr">
+        <is>
+          <t>16/04/2026</t>
+        </is>
+      </c>
+      <c r="B3550" s="2" t="n">
+        <v>-0.263763</v>
+      </c>
+    </row>
+    <row r="3551">
+      <c r="A3551" s="3" t="inlineStr">
+        <is>
+          <t>17/04/2026</t>
+        </is>
+      </c>
+      <c r="B3551" s="3" t="n">
+        <v>2.6081</v>
+      </c>
+    </row>
+    <row r="3552">
+      <c r="A3552" s="2" t="inlineStr">
+        <is>
+          <t>20/04/2026</t>
+        </is>
+      </c>
+      <c r="B3552" s="2" t="n">
+        <v>-0.997101</v>
+      </c>
+    </row>
+    <row r="3553">
+      <c r="A3553" s="3" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B3553" s="3" t="n">
+        <v>0.60559</v>
       </c>
     </row>
   </sheetData>
@@ -36019,27 +36059,27 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>1Y  (2025-04-15 to 2026-04-15)</t>
+          <t>1Y  (2025-04-21 to 2026-04-21)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>2Y  (2024-04-15 to 2026-04-15)</t>
+          <t>2Y  (2024-04-21 to 2026-04-21)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>3Y  (2023-04-15 to 2026-04-15)</t>
+          <t>3Y  (2023-04-21 to 2026-04-21)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>4Y  (2022-04-15 to 2026-04-15)</t>
+          <t>4Y  (2022-04-21 to 2026-04-21)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>5Y  (2021-04-15 to 2026-04-15)</t>
+          <t>5Y  (2021-04-21 to 2026-04-21)</t>
         </is>
       </c>
     </row>
@@ -36055,19 +36095,19 @@
         </is>
       </c>
       <c r="C2" s="5" t="n">
-        <v>18.0531</v>
+        <v>18.0603</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>15.8079</v>
+        <v>15.9557</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>14.029</v>
+        <v>14.1305</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>13.6893</v>
+        <v>13.7675</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>12.9754</v>
+        <v>13.0409</v>
       </c>
     </row>
     <row r="3">
@@ -36082,19 +36122,19 @@
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>17.9309</v>
+        <v>17.8927</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>16.0236</v>
+        <v>16.1358</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>14.1672</v>
+        <v>14.2598</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>13.6884</v>
+        <v>13.7609</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>13.0505</v>
+        <v>13.1108</v>
       </c>
     </row>
     <row r="5">
@@ -36109,19 +36149,19 @@
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>13.5222</v>
+        <v>11.3444</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>19.0689</v>
+        <v>19.8336</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>22.0542</v>
+        <v>22.8509</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>9.840400000000001</v>
+        <v>10.2069</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>10.2193</v>
+        <v>10.5136</v>
       </c>
     </row>
     <row r="6">
@@ -36136,19 +36176,19 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>23.7922</v>
+        <v>21.1634</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>33.7672</v>
+        <v>33.2522</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>34.7481</v>
+        <v>35.6593</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>20.8899</v>
+        <v>21.1969</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>20.9463</v>
+        <v>21.2515</v>
       </c>
     </row>
     <row r="8">
@@ -36163,19 +36203,19 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>0.621</v>
+        <v>0.5001</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>0.8875</v>
+        <v>0.9287</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.9876</v>
+        <v>1.0376</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>-0.0616</v>
+        <v>-0.0355</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>-0.1692</v>
+        <v>-0.1469</v>
       </c>
     </row>
     <row r="9">
@@ -36190,19 +36230,19 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>1.1979</v>
+        <v>1.0536</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>1.7929</v>
+        <v>1.7499</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>1.8739</v>
+        <v>1.9264</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>0.7456</v>
+        <v>0.7631</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>0.6538</v>
+        <v>0.6729000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -36244,19 +36284,19 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>0.9802999999999999</v>
+        <v>0.9779</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>0.997</v>
+        <v>0.9963</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>0.9846</v>
+        <v>0.9844000000000001</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>0.97</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>0.9724</v>
+        <v>0.9723000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -36298,19 +36338,19 @@
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>2.9045</v>
+        <v>2.8936</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>2.8901</v>
+        <v>2.7711</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>3.1531</v>
+        <v>3.1496</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>3.3492</v>
+        <v>3.3479</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>3.3529</v>
+        <v>3.3523</v>
       </c>
     </row>
     <row r="17">
@@ -36331,7 +36371,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="F17" s="5" t="n">
         <v>0</v>
@@ -36352,19 +36392,19 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>0.1049</v>
+        <v>0.1002</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>0.1474</v>
+        <v>0.1347</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>0.1291</v>
+        <v>0.1304</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>0.1102</v>
+        <v>0.1098</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>0.1067</v>
+        <v>0.1068</v>
       </c>
     </row>
     <row r="20">
@@ -36436,7 +36476,7 @@
         <v>1.5288</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>1.2823</v>
+        <v>1.2835</v>
       </c>
       <c r="E23" s="5" t="n">
         <v>1.1344</v>
@@ -36463,7 +36503,7 @@
         <v>1.541</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>1.2924</v>
+        <v>1.2933</v>
       </c>
       <c r="E24" s="7" t="n">
         <v>1.1507</v>
@@ -36541,19 +36581,19 @@
         </is>
       </c>
       <c r="C29" s="5" t="n">
-        <v>0.8929</v>
+        <v>0.7169</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>1.2727</v>
+        <v>1.3397</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>1.4739</v>
+        <v>1.5565</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>-0.0878</v>
+        <v>-0.0508</v>
       </c>
       <c r="G29" s="5" t="n">
-        <v>-0.2394</v>
+        <v>-0.2087</v>
       </c>
     </row>
     <row r="30">
@@ -36568,19 +36608,19 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>1.7699</v>
+        <v>1.5476</v>
       </c>
       <c r="D30" s="7" t="n">
-        <v>2.6576</v>
+        <v>2.6035</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>2.8842</v>
+        <v>2.9781</v>
       </c>
       <c r="F30" s="7" t="n">
-        <v>1.0935</v>
+        <v>1.1235</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>0.9507</v>
+        <v>0.9818</v>
       </c>
     </row>
   </sheetData>

</xml_diff>